<commit_message>
Added Baseclass and locators of login page, verify otp page and logout button
</commit_message>
<xml_diff>
--- a/epic_Shubhastro_QA/TestData/TestData.xlsx
+++ b/epic_Shubhastro_QA/TestData/TestData.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IN10\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E35014-BABA-4CDD-9B46-2D2D13CC88CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,12 +20,26 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="2">
+  <si>
+    <t>Test@123</t>
+  </si>
+  <si>
+    <t>59@yopmail.com</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -49,8 +69,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +351,39 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>7026868217</v>
+      </c>
+      <c r="B1">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>7026868217</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add login test suite: valid/invalid login, Max Device handling, empty-fields validation
- Robust Login button handling (presence + scroll + JS click)

- Route explicit waits through SeleniumUtility; add presence and non-throwing helpers

- Validate pass/fail with TestNG assertions; broaden error locator (invalid credentials / user not found)

- Valid login flow: profile icon then logout with scroll

- Handle Max Device limit page (MaxDeviceLimitPage POM): log out a device and continue

- Add empty-fields validation test; reset page in BeforeMethod for test independence

- Update test data and ignore run artifacts
</commit_message>
<xml_diff>
--- a/epic_Shubhastro_QA/TestData/TestData.xlsx
+++ b/epic_Shubhastro_QA/TestData/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IN10\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IN10\Desktop\Epic_Epicon\epic_Shubhastro_QA\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56FBD2BA-5F2C-4E6B-BF52-5E0760B46BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F6F65C-F89E-4F96-8E48-4333427E5531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Test@123</t>
   </si>
@@ -36,28 +36,35 @@
     <t>59@yopmail.com</t>
   </si>
   <si>
-    <t>58@yopmail.com</t>
-  </si>
-  <si>
     <t>Test@122</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>fail</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>expectedResult</t>
+  </si>
+  <si>
+    <t>5@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -80,17 +87,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -369,43 +372,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" t="s">
         <v>0</v>
       </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
+      <c r="C4" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{E87996E0-0A5F-49C5-9503-136499527675}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{F02D1E34-8A76-48AA-882B-44BF6770AD4F}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{B1247E0F-A039-45DA-A4DE-8EFDDC603007}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>